<commit_message>
chore(data): sync FEB data 2026-05-11 09:58
</commit_message>
<xml_diff>
--- a/data/1FEB_25_26/clutch_aggregated_25_26_1FEB.xlsx
+++ b/data/1FEB_25_26/clutch_aggregated_25_26_1FEB.xlsx
@@ -557,13 +557,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" t="n">
-        <v>22.52</v>
+        <v>22.89</v>
       </c>
       <c r="E2" t="n">
-        <v>1351.2</v>
+        <v>1373.4</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -611,13 +611,13 @@
         <v>6</v>
       </c>
       <c r="U2" t="n">
-        <v>14.9045026642984</v>
+        <v>14.66358235037134</v>
       </c>
       <c r="V2" t="n">
-        <v>-7</v>
+        <v>-9</v>
       </c>
       <c r="W2" t="n">
-        <v>-0.6147957371225573</v>
+        <v>-2.221284403669724</v>
       </c>
     </row>
     <row r="3">
@@ -707,25 +707,25 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D4" t="n">
-        <v>19.81</v>
+        <v>24.51</v>
       </c>
       <c r="E4" t="n">
-        <v>1188.6</v>
+        <v>1470.6</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H4" t="n">
         <v>1</v>
       </c>
       <c r="I4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J4" t="n">
         <v>1</v>
@@ -737,13 +737,13 @@
         <v>2</v>
       </c>
       <c r="M4" t="n">
-        <v>0.375</v>
+        <v>0.3</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P4" t="n">
         <v>0</v>
@@ -761,13 +761,13 @@
         <v>3</v>
       </c>
       <c r="U4" t="n">
-        <v>20.16330641090358</v>
+        <v>19.13292941656466</v>
       </c>
       <c r="V4" t="n">
         <v>-7</v>
       </c>
       <c r="W4" t="n">
-        <v>-7.023528520949016</v>
+        <v>-1.27968584251326</v>
       </c>
     </row>
     <row r="5">
@@ -932,25 +932,25 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D7" t="n">
-        <v>40.17</v>
+        <v>44.87</v>
       </c>
       <c r="E7" t="n">
-        <v>2410.2</v>
+        <v>2692.2</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H7" t="n">
         <v>5</v>
       </c>
       <c r="I7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="J7" t="n">
         <v>2</v>
@@ -962,7 +962,7 @@
         <v>2</v>
       </c>
       <c r="M7" t="n">
-        <v>0.5</v>
+        <v>0.4615384615384616</v>
       </c>
       <c r="N7" t="n">
         <v>0</v>
@@ -977,22 +977,22 @@
         <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="S7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="T7" t="n">
         <v>8</v>
       </c>
       <c r="U7" t="n">
-        <v>20.31510082150859</v>
+        <v>19.73636282594161</v>
       </c>
       <c r="V7" t="n">
         <v>-3</v>
       </c>
       <c r="W7" t="n">
-        <v>5.355354742345035</v>
+        <v>7.196246935591711</v>
       </c>
     </row>
     <row r="8">
@@ -1157,37 +1157,37 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D10" t="n">
-        <v>36.41</v>
+        <v>41.11</v>
       </c>
       <c r="E10" t="n">
-        <v>2184.6</v>
+        <v>2466.6</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="H10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I10" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J10" t="n">
         <v>2</v>
       </c>
       <c r="K10" t="n">
+        <v>19</v>
+      </c>
+      <c r="L10" t="n">
         <v>17</v>
       </c>
-      <c r="L10" t="n">
-        <v>16</v>
-      </c>
       <c r="M10" t="n">
-        <v>0.32</v>
+        <v>0.3103448275862069</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
@@ -1202,22 +1202,22 @@
         <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S10" t="n">
         <v>5</v>
       </c>
       <c r="T10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="U10" t="n">
-        <v>62.35842351002474</v>
+        <v>63.48244222816834</v>
       </c>
       <c r="V10" t="n">
         <v>-2</v>
       </c>
       <c r="W10" t="n">
-        <v>-0.9339686899203524</v>
+        <v>1.794337144247141</v>
       </c>
     </row>
     <row r="11">
@@ -1307,13 +1307,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D12" t="n">
-        <v>25.79</v>
+        <v>30.12</v>
       </c>
       <c r="E12" t="n">
-        <v>1547.4</v>
+        <v>1807.2</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
@@ -1331,10 +1331,10 @@
         <v>2</v>
       </c>
       <c r="K12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M12" t="n">
         <v>0.8</v>
@@ -1352,22 +1352,22 @@
         <v>1</v>
       </c>
       <c r="R12" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T12" t="n">
         <v>2</v>
       </c>
       <c r="U12" t="n">
-        <v>12.95260566110896</v>
+        <v>13.28718791500664</v>
       </c>
       <c r="V12" t="n">
-        <v>-8</v>
+        <v>-6</v>
       </c>
       <c r="W12" t="n">
-        <v>-33.5263823187282</v>
+        <v>-22.91610225763613</v>
       </c>
     </row>
     <row r="13">
@@ -1382,28 +1382,28 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D13" t="n">
-        <v>44.89</v>
+        <v>49.59</v>
       </c>
       <c r="E13" t="n">
-        <v>2693.4</v>
+        <v>2975.4</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="H13" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="I13" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K13" t="n">
         <v>6</v>
@@ -1412,7 +1412,7 @@
         <v>4</v>
       </c>
       <c r="M13" t="n">
-        <v>0.75</v>
+        <v>0.8214285714285714</v>
       </c>
       <c r="N13" t="n">
         <v>0</v>
@@ -1427,22 +1427,22 @@
         <v>5</v>
       </c>
       <c r="R13" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S13" t="n">
         <v>8</v>
       </c>
       <c r="T13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U13" t="n">
-        <v>25.17963911784362</v>
+        <v>25.59764065335754</v>
       </c>
       <c r="V13" t="n">
         <v>0</v>
       </c>
       <c r="W13" t="n">
-        <v>7.059685898863886</v>
+        <v>8.563829401088926</v>
       </c>
     </row>
     <row r="14">
@@ -2432,13 +2432,13 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D27" t="n">
-        <v>0.53</v>
+        <v>2.05</v>
       </c>
       <c r="E27" t="n">
-        <v>31.8</v>
+        <v>123</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -2489,10 +2489,10 @@
         <v>0</v>
       </c>
       <c r="V27" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="W27" t="n">
-        <v>-71.69811320754717</v>
+        <v>-78.71375609756099</v>
       </c>
     </row>
     <row r="28">
@@ -2507,22 +2507,22 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D28" t="n">
-        <v>6.8</v>
+        <v>11.5</v>
       </c>
       <c r="E28" t="n">
-        <v>408</v>
+        <v>690</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
       </c>
       <c r="G28" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I28" t="n">
         <v>0</v>
@@ -2537,7 +2537,7 @@
         <v>3</v>
       </c>
       <c r="M28" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8</v>
       </c>
       <c r="N28" t="n">
         <v>0</v>
@@ -2561,13 +2561,13 @@
         <v>0</v>
       </c>
       <c r="U28" t="n">
-        <v>26.52155882352941</v>
+        <v>25.89970434782609</v>
       </c>
       <c r="V28" t="n">
         <v>-8</v>
       </c>
       <c r="W28" t="n">
-        <v>-163.0636617647058</v>
+        <v>-105.7916434782609</v>
       </c>
     </row>
     <row r="29">
@@ -2657,19 +2657,19 @@
         </is>
       </c>
       <c r="C30" t="n">
+        <v>13</v>
+      </c>
+      <c r="D30" t="n">
+        <v>37.87</v>
+      </c>
+      <c r="E30" t="n">
+        <v>2272.2</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
         <v>12</v>
-      </c>
-      <c r="D30" t="n">
-        <v>34.69</v>
-      </c>
-      <c r="E30" t="n">
-        <v>2081.4</v>
-      </c>
-      <c r="F30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" t="n">
-        <v>11</v>
       </c>
       <c r="H30" t="n">
         <v>2</v>
@@ -2687,7 +2687,7 @@
         <v>4</v>
       </c>
       <c r="M30" t="n">
-        <v>0.2272727272727273</v>
+        <v>0.2083333333333333</v>
       </c>
       <c r="N30" t="n">
         <v>0</v>
@@ -2711,13 +2711,13 @@
         <v>0</v>
       </c>
       <c r="U30" t="n">
-        <v>30.09992216777169</v>
+        <v>29.67167414840243</v>
       </c>
       <c r="V30" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="W30" t="n">
-        <v>-5.448466416834818</v>
+        <v>-2.891663585951937</v>
       </c>
     </row>
     <row r="31">
@@ -2732,44 +2732,44 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D31" t="n">
-        <v>26.96</v>
+        <v>31.66</v>
       </c>
       <c r="E31" t="n">
-        <v>1617.6</v>
+        <v>1899.6</v>
       </c>
       <c r="F31" t="n">
         <v>0</v>
       </c>
       <c r="G31" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H31" t="n">
         <v>6</v>
       </c>
       <c r="I31" t="n">
+        <v>7</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" t="n">
+        <v>3</v>
+      </c>
+      <c r="L31" t="n">
+        <v>1</v>
+      </c>
+      <c r="M31" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N31" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" t="n">
         <v>6</v>
       </c>
-      <c r="J31" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" t="n">
-        <v>3</v>
-      </c>
-      <c r="L31" t="n">
-        <v>1</v>
-      </c>
-      <c r="M31" t="n">
-        <v>0.3529411764705883</v>
-      </c>
-      <c r="N31" t="n">
-        <v>0</v>
-      </c>
-      <c r="O31" t="n">
-        <v>4</v>
-      </c>
       <c r="P31" t="n">
         <v>1</v>
       </c>
@@ -2777,22 +2777,22 @@
         <v>1</v>
       </c>
       <c r="R31" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="S31" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="U31" t="n">
-        <v>46.97092729970326</v>
+        <v>41.85363866077068</v>
       </c>
       <c r="V31" t="n">
         <v>0</v>
       </c>
       <c r="W31" t="n">
-        <v>-15.55140207715134</v>
+        <v>-16.64677195198989</v>
       </c>
     </row>
     <row r="32">
@@ -2882,67 +2882,67 @@
         </is>
       </c>
       <c r="C33" t="n">
+        <v>6</v>
+      </c>
+      <c r="D33" t="n">
+        <v>12.21</v>
+      </c>
+      <c r="E33" t="n">
+        <v>732.6</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
+        <v>8</v>
+      </c>
+      <c r="H33" t="n">
+        <v>4</v>
+      </c>
+      <c r="I33" t="n">
+        <v>4</v>
+      </c>
+      <c r="J33" t="n">
+        <v>1</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" t="n">
+        <v>0.5625</v>
+      </c>
+      <c r="N33" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" t="n">
+        <v>1</v>
+      </c>
+      <c r="P33" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" t="n">
         <v>5</v>
       </c>
-      <c r="D33" t="n">
-        <v>7.51</v>
-      </c>
-      <c r="E33" t="n">
-        <v>450.6</v>
-      </c>
-      <c r="F33" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" t="n">
-        <v>5</v>
-      </c>
-      <c r="H33" t="n">
-        <v>3</v>
-      </c>
-      <c r="I33" t="n">
-        <v>2</v>
-      </c>
-      <c r="J33" t="n">
-        <v>1</v>
-      </c>
-      <c r="K33" t="n">
-        <v>0</v>
-      </c>
-      <c r="L33" t="n">
-        <v>0</v>
-      </c>
-      <c r="M33" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="N33" t="n">
-        <v>0</v>
-      </c>
-      <c r="O33" t="n">
-        <v>0</v>
-      </c>
-      <c r="P33" t="n">
-        <v>2</v>
-      </c>
-      <c r="Q33" t="n">
-        <v>0</v>
-      </c>
-      <c r="R33" t="n">
-        <v>4</v>
-      </c>
       <c r="S33" t="n">
         <v>3</v>
       </c>
       <c r="T33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U33" t="n">
-        <v>69.36014647137151</v>
+        <v>57.09620802620803</v>
       </c>
       <c r="V33" t="n">
         <v>3</v>
       </c>
       <c r="W33" t="n">
-        <v>64.70936085219707</v>
+        <v>30.97430794430795</v>
       </c>
     </row>
     <row r="34">
@@ -3257,67 +3257,67 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D38" t="n">
-        <v>31.27</v>
+        <v>35.97</v>
       </c>
       <c r="E38" t="n">
-        <v>1876.2</v>
+        <v>2158.2</v>
       </c>
       <c r="F38" t="n">
         <v>0</v>
       </c>
       <c r="G38" t="n">
+        <v>11</v>
+      </c>
+      <c r="H38" t="n">
+        <v>9</v>
+      </c>
+      <c r="I38" t="n">
+        <v>2</v>
+      </c>
+      <c r="J38" t="n">
+        <v>2</v>
+      </c>
+      <c r="K38" t="n">
+        <v>2</v>
+      </c>
+      <c r="L38" t="n">
+        <v>2</v>
+      </c>
+      <c r="M38" t="n">
+        <v>0.9090909090909091</v>
+      </c>
+      <c r="N38" t="n">
+        <v>0</v>
+      </c>
+      <c r="O38" t="n">
+        <v>1</v>
+      </c>
+      <c r="P38" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>2</v>
+      </c>
+      <c r="R38" t="n">
+        <v>14</v>
+      </c>
+      <c r="S38" t="n">
+        <v>6</v>
+      </c>
+      <c r="T38" t="n">
         <v>8</v>
       </c>
-      <c r="H38" t="n">
-        <v>7</v>
-      </c>
-      <c r="I38" t="n">
-        <v>2</v>
-      </c>
-      <c r="J38" t="n">
-        <v>2</v>
-      </c>
-      <c r="K38" t="n">
-        <v>2</v>
-      </c>
-      <c r="L38" t="n">
-        <v>2</v>
-      </c>
-      <c r="M38" t="n">
-        <v>1</v>
-      </c>
-      <c r="N38" t="n">
-        <v>0</v>
-      </c>
-      <c r="O38" t="n">
-        <v>0</v>
-      </c>
-      <c r="P38" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q38" t="n">
-        <v>2</v>
-      </c>
-      <c r="R38" t="n">
-        <v>11</v>
-      </c>
-      <c r="S38" t="n">
-        <v>5</v>
-      </c>
-      <c r="T38" t="n">
-        <v>6</v>
-      </c>
       <c r="U38" t="n">
-        <v>13.74765909817717</v>
+        <v>16.8512454823464</v>
       </c>
       <c r="V38" t="n">
         <v>11</v>
       </c>
       <c r="W38" t="n">
-        <v>27.5089958426607</v>
+        <v>20.91841256602725</v>
       </c>
     </row>
     <row r="39">
@@ -5207,22 +5207,22 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D64" t="n">
-        <v>18.36</v>
+        <v>20.43</v>
       </c>
       <c r="E64" t="n">
-        <v>1101.6</v>
+        <v>1225.8</v>
       </c>
       <c r="F64" t="n">
         <v>0</v>
       </c>
       <c r="G64" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="H64" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I64" t="n">
         <v>0</v>
@@ -5243,7 +5243,7 @@
         <v>0</v>
       </c>
       <c r="O64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P64" t="n">
         <v>0</v>
@@ -5261,13 +5261,13 @@
         <v>4</v>
       </c>
       <c r="U64" t="n">
-        <v>25.02211328976034</v>
+        <v>29.24194322075379</v>
       </c>
       <c r="V64" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="W64" t="n">
-        <v>79.27154684095861</v>
+        <v>71.85363680861478</v>
       </c>
     </row>
     <row r="65">
@@ -5357,13 +5357,13 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D66" t="n">
-        <v>27</v>
+        <v>27.08</v>
       </c>
       <c r="E66" t="n">
-        <v>1620</v>
+        <v>1624.8</v>
       </c>
       <c r="F66" t="n">
         <v>0</v>
@@ -5411,13 +5411,13 @@
         <v>5</v>
       </c>
       <c r="U66" t="n">
-        <v>17.96831111111111</v>
+        <v>17.91522895125554</v>
       </c>
       <c r="V66" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="W66" t="n">
-        <v>93.39345185185185</v>
+        <v>93.11754800590842</v>
       </c>
     </row>
     <row r="67">
@@ -5432,13 +5432,13 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D67" t="n">
-        <v>17.88</v>
+        <v>19.95</v>
       </c>
       <c r="E67" t="n">
-        <v>1072.8</v>
+        <v>1197</v>
       </c>
       <c r="F67" t="n">
         <v>0</v>
@@ -5468,7 +5468,7 @@
         <v>0</v>
       </c>
       <c r="O67" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P67" t="n">
         <v>1</v>
@@ -5486,13 +5486,13 @@
         <v>0</v>
       </c>
       <c r="U67" t="n">
-        <v>16.95011744966443</v>
+        <v>15.19138345864662</v>
       </c>
       <c r="V67" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="W67" t="n">
-        <v>-18.90921700223714</v>
+        <v>-16.31842606516291</v>
       </c>
     </row>
     <row r="68">
@@ -5582,13 +5582,13 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D69" t="n">
-        <v>12.84</v>
+        <v>12.92</v>
       </c>
       <c r="E69" t="n">
-        <v>770.4</v>
+        <v>775.1999999999999</v>
       </c>
       <c r="F69" t="n">
         <v>0</v>
@@ -5636,13 +5636,13 @@
         <v>3</v>
       </c>
       <c r="U69" t="n">
-        <v>14.92002336448598</v>
+        <v>14.82763931888545</v>
       </c>
       <c r="V69" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="W69" t="n">
-        <v>23.99939252336448</v>
+        <v>23.85078947368421</v>
       </c>
     </row>
     <row r="70">
@@ -5657,22 +5657,22 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D70" t="n">
-        <v>19.82</v>
+        <v>21.8</v>
       </c>
       <c r="E70" t="n">
-        <v>1189.2</v>
+        <v>1308</v>
       </c>
       <c r="F70" t="n">
         <v>0</v>
       </c>
       <c r="G70" t="n">
+        <v>6</v>
+      </c>
+      <c r="H70" t="n">
         <v>5</v>
-      </c>
-      <c r="H70" t="n">
-        <v>4</v>
       </c>
       <c r="I70" t="n">
         <v>0</v>
@@ -5687,7 +5687,7 @@
         <v>8</v>
       </c>
       <c r="M70" t="n">
-        <v>0.8</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="N70" t="n">
         <v>0</v>
@@ -5702,22 +5702,22 @@
         <v>0</v>
       </c>
       <c r="R70" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S70" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T70" t="n">
         <v>5</v>
       </c>
       <c r="U70" t="n">
-        <v>30.28271442986882</v>
+        <v>32.07355045871559</v>
       </c>
       <c r="V70" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="W70" t="n">
-        <v>63.77890010090817</v>
+        <v>55.50932110091743</v>
       </c>
     </row>
     <row r="71">
@@ -5807,28 +5807,28 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D72" t="n">
-        <v>4.13</v>
+        <v>6.199999999999999</v>
       </c>
       <c r="E72" t="n">
-        <v>247.8</v>
+        <v>372</v>
       </c>
       <c r="F72" t="n">
         <v>0</v>
       </c>
       <c r="G72" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H72" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I72" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J72" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K72" t="n">
         <v>0</v>
@@ -5837,7 +5837,7 @@
         <v>0</v>
       </c>
       <c r="M72" t="n">
-        <v>0.5</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="N72" t="n">
         <v>0</v>
@@ -5861,13 +5861,13 @@
         <v>0</v>
       </c>
       <c r="U72" t="n">
-        <v>21.13133171912833</v>
+        <v>25.20411290322581</v>
       </c>
       <c r="V72" t="n">
-        <v>-1</v>
+        <v>-2</v>
       </c>
       <c r="W72" t="n">
-        <v>-91.80847457627119</v>
+        <v>-59.13303225806453</v>
       </c>
     </row>
     <row r="73">
@@ -6032,25 +6032,25 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D75" t="n">
-        <v>22.15</v>
+        <v>24.13</v>
       </c>
       <c r="E75" t="n">
-        <v>1329</v>
+        <v>1447.8</v>
       </c>
       <c r="F75" t="n">
         <v>0</v>
       </c>
       <c r="G75" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H75" t="n">
         <v>4</v>
       </c>
       <c r="I75" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J75" t="n">
         <v>1</v>
@@ -6062,7 +6062,7 @@
         <v>6</v>
       </c>
       <c r="M75" t="n">
-        <v>0.3461538461538461</v>
+        <v>0.3214285714285715</v>
       </c>
       <c r="N75" t="n">
         <v>0</v>
@@ -6077,22 +6077,22 @@
         <v>0</v>
       </c>
       <c r="R75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S75" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T75" t="n">
         <v>0</v>
       </c>
       <c r="U75" t="n">
-        <v>48.37629796839729</v>
+        <v>48.50953170327394</v>
       </c>
       <c r="V75" t="n">
-        <v>2</v>
+        <v>-2</v>
       </c>
       <c r="W75" t="n">
-        <v>27.98348081264108</v>
+        <v>23.44962702030668</v>
       </c>
     </row>
     <row r="76">
@@ -15557,13 +15557,13 @@
         </is>
       </c>
       <c r="C202" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D202" t="n">
-        <v>2.4</v>
+        <v>2.48</v>
       </c>
       <c r="E202" t="n">
-        <v>144</v>
+        <v>148.8</v>
       </c>
       <c r="F202" t="n">
         <v>0</v>
@@ -15614,10 +15614,10 @@
         <v>0</v>
       </c>
       <c r="V202" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="W202" t="n">
-        <v>-5.870416666666665</v>
+        <v>-5.681048387096772</v>
       </c>
     </row>
     <row r="203">
@@ -15707,13 +15707,13 @@
         </is>
       </c>
       <c r="C204" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D204" t="n">
-        <v>1.98</v>
+        <v>2.56</v>
       </c>
       <c r="E204" t="n">
-        <v>118.8</v>
+        <v>153.6</v>
       </c>
       <c r="F204" t="n">
         <v>0</v>
@@ -15761,13 +15761,13 @@
         <v>1</v>
       </c>
       <c r="U204" t="n">
-        <v>22.68</v>
+        <v>17.5415625</v>
       </c>
       <c r="V204" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="W204" t="n">
-        <v>-40.97999999999999</v>
+        <v>-31.69546875</v>
       </c>
     </row>
     <row r="205">
@@ -15782,13 +15782,13 @@
         </is>
       </c>
       <c r="C205" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D205" t="n">
-        <v>35.09</v>
+        <v>37.16</v>
       </c>
       <c r="E205" t="n">
-        <v>2105.4</v>
+        <v>2229.6</v>
       </c>
       <c r="F205" t="n">
         <v>0</v>
@@ -15806,10 +15806,10 @@
         <v>0</v>
       </c>
       <c r="K205" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L205" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M205" t="n">
         <v>0.1538461538461539</v>
@@ -15836,13 +15836,13 @@
         <v>5</v>
       </c>
       <c r="U205" t="n">
-        <v>49.45485893416929</v>
+        <v>48.09259956942951</v>
       </c>
       <c r="V205" t="n">
-        <v>-12</v>
+        <v>-11</v>
       </c>
       <c r="W205" t="n">
-        <v>-30.82259618124822</v>
+        <v>-29.4431942949408</v>
       </c>
     </row>
     <row r="206">
@@ -16082,13 +16082,13 @@
         </is>
       </c>
       <c r="C209" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D209" t="n">
-        <v>2.03</v>
+        <v>3.43</v>
       </c>
       <c r="E209" t="n">
-        <v>121.8</v>
+        <v>205.8</v>
       </c>
       <c r="F209" t="n">
         <v>0</v>
@@ -16136,13 +16136,13 @@
         <v>0</v>
       </c>
       <c r="U209" t="n">
-        <v>32.15448275862069</v>
+        <v>19.03020408163265</v>
       </c>
       <c r="V209" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="W209" t="n">
-        <v>30.10778325123152</v>
+        <v>28.94950437317784</v>
       </c>
     </row>
     <row r="210">
@@ -16157,25 +16157,25 @@
         </is>
       </c>
       <c r="C210" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D210" t="n">
-        <v>12.82</v>
+        <v>14.89</v>
       </c>
       <c r="E210" t="n">
-        <v>769.2</v>
+        <v>893.4</v>
       </c>
       <c r="F210" t="n">
         <v>0</v>
       </c>
       <c r="G210" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H210" t="n">
         <v>3</v>
       </c>
       <c r="I210" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J210" t="n">
         <v>1</v>
@@ -16187,7 +16187,7 @@
         <v>3</v>
       </c>
       <c r="M210" t="n">
-        <v>0.5833333333333334</v>
+        <v>0.5</v>
       </c>
       <c r="N210" t="n">
         <v>0</v>
@@ -16202,22 +16202,22 @@
         <v>2</v>
       </c>
       <c r="R210" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S210" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T210" t="n">
         <v>0</v>
       </c>
       <c r="U210" t="n">
-        <v>30.49762090483619</v>
+        <v>30.20740094022834</v>
       </c>
       <c r="V210" t="n">
-        <v>-19</v>
+        <v>-18</v>
       </c>
       <c r="W210" t="n">
-        <v>-49.04762870514821</v>
+        <v>-43.07151108126259</v>
       </c>
     </row>
     <row r="211">
@@ -16307,13 +16307,13 @@
         </is>
       </c>
       <c r="C212" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D212" t="n">
-        <v>1.51</v>
+        <v>3.58</v>
       </c>
       <c r="E212" t="n">
-        <v>90.59999999999999</v>
+        <v>214.8</v>
       </c>
       <c r="F212" t="n">
         <v>0</v>
@@ -16331,10 +16331,10 @@
         <v>0</v>
       </c>
       <c r="K212" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L212" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M212" t="n">
         <v>1</v>
@@ -16361,13 +16361,13 @@
         <v>0</v>
       </c>
       <c r="U212" t="n">
-        <v>14.34735099337748</v>
+        <v>20.50684357541899</v>
       </c>
       <c r="V212" t="n">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="W212" t="n">
-        <v>-10.90013245033112</v>
+        <v>-8.101508379888267</v>
       </c>
     </row>
     <row r="213">
@@ -16382,13 +16382,13 @@
         </is>
       </c>
       <c r="C213" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D213" t="n">
-        <v>11.57</v>
+        <v>12.97</v>
       </c>
       <c r="E213" t="n">
-        <v>694.2</v>
+        <v>778.2</v>
       </c>
       <c r="F213" t="n">
         <v>0</v>
@@ -16406,10 +16406,10 @@
         <v>0</v>
       </c>
       <c r="K213" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="L213" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="M213" t="n">
         <v>0</v>
@@ -16436,13 +16436,13 @@
         <v>1</v>
       </c>
       <c r="U213" t="n">
-        <v>19.7200691443388</v>
+        <v>24.78791056283731</v>
       </c>
       <c r="V213" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="W213" t="n">
-        <v>29.02229040622299</v>
+        <v>28.83314572089437</v>
       </c>
     </row>
     <row r="214">
@@ -16457,13 +16457,13 @@
         </is>
       </c>
       <c r="C214" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D214" t="n">
-        <v>24.71</v>
+        <v>24.79</v>
       </c>
       <c r="E214" t="n">
-        <v>1482.6</v>
+        <v>1487.4</v>
       </c>
       <c r="F214" t="n">
         <v>0</v>
@@ -16511,13 +16511,13 @@
         <v>1</v>
       </c>
       <c r="U214" t="n">
-        <v>11.60048968029138</v>
+        <v>11.56305365066559</v>
       </c>
       <c r="V214" t="n">
-        <v>2</v>
+        <v>-1</v>
       </c>
       <c r="W214" t="n">
-        <v>-11.7873452043707</v>
+        <v>-11.74930617184348</v>
       </c>
     </row>
     <row r="215">

</xml_diff>